<commit_message>
feat(F-NAR-019): TREE-AUT-007 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-007.xlsx
+++ b/stories/arbres/TREE-AUT-007.xlsx
@@ -2339,17 +2339,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le t-shirt, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton d'abord, ensuite la poignée. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?</t>
+          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le t-shirt, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton te tient le bras, attends. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis level="moderate"&gt;t-shirt&lt;/emphasis&gt;, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton d'abord, ensuite la poignée. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis level="moderate"&gt;t-shirt&lt;/emphasis&gt;, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton te tient le bras, attends. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis&gt;t-shirt&lt;/emphasis&gt;, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton d'abord, ensuite la poignée. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis&gt;t-shirt&lt;/emphasis&gt;, le coton froid. Je le mets, et je tire ! Elle enfile trop vite, une manche se coince. Son épaule reste coincée, comme le volet. Sors le bras, sans tirer le bois. Le coton te tient le bras, attends. La manche me tient ! Elle ralentit, et le bras passe, tout net. Le t-shirt sent le soleil, contre sa peau. Tu peux pousser, avec l'épaule. J'ai le coton, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2493,7 +2493,7 @@
 narrateur|Elle enfile trop vite, une manche se coince.
 narrateur|Son épaule reste coincée, comme le volet.
 papa|Sors le bras, sans tirer le bois.
-maman|Le coton d'abord, ensuite la poignée.
+maman|Le coton te tient le bras, attends.
 enfant-f|La manche me tient !
 narrateur|Elle ralentit, et le bras passe, tout net.
 narrateur|Le t-shirt sent le soleil, contre sa peau.
@@ -2912,17 +2912,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le volet a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. L'oiseau de papier dort dans le sac, face à la rue.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le volet a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Le sac a pris le soleil, toi. L'oiseau de papier dort dans le sac, face à la rue.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. L'oiseau de papier dort dans le sac, face à la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Le sac a pris le soleil, toi. L'oiseau de papier dort dans le sac, face à la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le &lt;emphasis&gt;volet&lt;/emphasis&gt; a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. L'oiseau de papier dort dans le sac, face à la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le sac, et le &lt;emphasis&gt;volet&lt;/emphasis&gt; a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Le sac a pris le soleil, toi. L'oiseau de papier dort dans le sac, face à la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3065,7 +3065,7 @@
 enfant-f|J'ai mis le t-shirt, le sac, et le volet a ouvert.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le sac a pris le soleil, toi.
 narrateur|L'oiseau de papier dort dans le sac, face à la rue.</t>
         </is>
       </c>
@@ -3283,17 +3283,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Un carré de soleil tient sur le manteau, près du bois ouvert.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Le vent est entré dans tes manches. Un carré de soleil tient sur le manteau, près du bois ouvert.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Un carré de soleil tient sur le manteau, près du bois ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Le vent est entré dans tes manches. Un carré de soleil tient sur le manteau, près du bois ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Un carré de soleil tient sur le manteau, près du bois ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le manteau, et le vent est entré. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Le vent est entré dans tes manches. Un carré de soleil tient sur le manteau, près du bois ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3432,7 +3432,7 @@
 enfant-f|J'ai mis le t-shirt, le manteau, et le vent est entré.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le vent est entré dans tes manches.
 narrateur|Un carré de soleil tient sur le manteau, près du bois ouvert.</t>
         </is>
       </c>
@@ -3650,17 +3650,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou regarde la rue, le menton sur la latte.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le doudou a gardé la latte. Le doudou regarde la rue, le menton sur la latte.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou regarde la rue, le menton sur la latte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le doudou a gardé la latte. Le doudou regarde la rue, le menton sur la latte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou regarde la rue, le menton sur la latte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le t-shirt, le doudou a vu la rue. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le doudou a gardé la latte. Le doudou regarde la rue, le menton sur la latte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3799,7 +3799,7 @@
 enfant-f|J'ai mis le t-shirt, le doudou a vu la rue.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le doudou a gardé la latte.
 narrateur|Le doudou regarde la rue, le menton sur la latte.</t>
         </is>
       </c>
@@ -3832,17 +3832,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les chaussettes, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Une chaussette, puis l'autre, sans sauter. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?</t>
+          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les chaussettes, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Assieds-toi, le parquet est trop lisse. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les &lt;emphasis level="moderate"&gt;chaussettes&lt;/emphasis&gt;, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Une chaussette, puis l'autre, sans sauter. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les &lt;emphasis level="moderate"&gt;chaussettes&lt;/emphasis&gt;, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Assieds-toi, le parquet est trop lisse. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les &lt;emphasis&gt;chaussettes&lt;/emphasis&gt;, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Une chaussette, puis l'autre, sans sauter. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend les &lt;emphasis&gt;chaussettes&lt;/emphasis&gt;, un peu froides. Je les mets, et je grimpe ! Elle enfile une seule, et court au tabouret. Le pied nu glisse sur le parquet, trop lisse. Les deux pieds, sinon le tabouret part. Assieds-toi, le parquet est trop lisse. J'ai failli tomber ! Elle s'assoit, et la deuxième chaussette passe. Le parquet n'attrape plus ses talons. Tu peux grimper, sans glisser. J'ai les deux, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3986,7 +3986,7 @@
 narrateur|Elle enfile une seule, et court au tabouret.
 narrateur|Le pied nu glisse sur le parquet, trop lisse.
 papa|Les deux pieds, sinon le tabouret part.
-maman|Une chaussette, puis l'autre, sans sauter.
+maman|Assieds-toi, le parquet est trop lisse.
 enfant-f|J'ai failli tomber !
 narrateur|Elle s'assoit, et la deuxième chaussette passe.
 narrateur|Le parquet n'attrape plus ses talons.
@@ -4404,17 +4404,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette garde un peu de parquet, sous le sac ouvert.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tes pieds n'ont pas glissé, sur le bois. Une chaussette garde un peu de parquet, sous le sac ouvert.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette garde un peu de parquet, sous le sac ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tes pieds n'ont pas glissé, sur le bois. Une chaussette garde un peu de parquet, sous le sac ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette garde un peu de parquet, sous le sac ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le sac, et j'ai grimpé. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tes pieds n'ont pas glissé, sur le bois. Une chaussette garde un peu de parquet, sous le sac ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4553,7 +4553,7 @@
 enfant-f|J'ai mis les chaussettes, le sac, et j'ai grimpé.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Tes pieds n'ont pas glissé, sur le bois.
 narrateur|Une chaussette garde un peu de parquet, sous le sac ouvert.</t>
         </is>
       </c>
@@ -4770,17 +4770,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près des chaussettes, sent le pain et le vent.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu pourras descendre, le manteau est prêt. Le manteau, près des chaussettes, sent le pain et le vent.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près des chaussettes, sent le pain et le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu pourras descendre, le manteau est prêt. Le manteau, près des chaussettes, sent le pain et le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près des chaussettes, sent le pain et le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le manteau, sans glisser. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu pourras descendre, le manteau est prêt. Le manteau, près des chaussettes, sent le pain et le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4919,7 +4919,7 @@
 enfant-f|J'ai mis les chaussettes, le manteau, sans glisser.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Tu pourras descendre, le manteau est prêt.
 narrateur|Le manteau, près des chaussettes, sent le pain et le vent.</t>
         </is>
       </c>
@@ -5136,17 +5136,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, assis sur une chaussette, voit le moineau.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le tabouret est resté droit, lui. Le doudou, assis sur une chaussette, voit le moineau.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, assis sur une chaussette, voit le moineau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le tabouret est resté droit, lui. Le doudou, assis sur une chaussette, voit le moineau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, assis sur une chaussette, voit le moineau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis les chaussettes, le doudou sur le tabouret. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Le tabouret est resté droit, lui. Le doudou, assis sur une chaussette, voit le moineau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5285,7 +5285,7 @@
 enfant-f|J'ai mis les chaussettes, le doudou sur le tabouret.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le tabouret est resté droit, lui.
 narrateur|Le doudou, assis sur une chaussette, voit le moineau.</t>
         </is>
       </c>
@@ -5318,17 +5318,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le gilet, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton d'abord, ensuite le bois. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?</t>
+          <t>Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le gilet, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton a sauté, le bois peut attendre. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton d'abord, ensuite le bois. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton a sauté, le bois peut attendre. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton d'abord, ensuite le bois. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans la chambre, le volet reste coincé, trop lourd. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, la laine un peu rêche. Je le mets, et je pousse ! Elle enfile trop vite, un bouton saute. La poignée froide lui pique la paume, trop nue. Le bouton a sauté, le bois peut attendre. La laine tiédit tes épaules, et tes mains. Le bouton m'a échappé ! Elle le retrouve, sous la chaise, sans courir. Le gilet ferme, et la poche attend, vide. Tu peux pousser, l'épaule au chaud. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5471,7 +5471,7 @@
 enfant-f|Je le mets, et je pousse !
 narrateur|Elle enfile trop vite, un bouton saute.
 narrateur|La poignée froide lui pique la paume, trop nue.
-papa|Le bouton d'abord, ensuite le bois.
+papa|Le bouton a sauté, le bois peut attendre.
 maman|La laine tiédit tes épaules, et tes mains.
 enfant-f|Le bouton m'a échappé !
 narrateur|Elle le retrouve, sous la chaise, sans courir.
@@ -5890,17 +5890,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet garde une plume, collée au sac.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. La poche a gardé l'oiseau, au chaud. La poche du gilet garde une plume, collée au sac.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet garde une plume, collée au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. La poche a gardé l'oiseau, au chaud. La poche du gilet garde une plume, collée au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet garde une plume, collée au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le sac dans la poche, et ça a ouvert. Sur la chaise de la chambre, le linge s'est tu. À table, le pain casse, tiède, sous les doigts. La poche a gardé l'oiseau, au chaud. La poche du gilet garde une plume, collée au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6039,7 +6039,7 @@
 enfant-f|J'ai mis le gilet, le sac dans la poche, et ça a ouvert.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|La poche a gardé l'oiseau, au chaud.
 narrateur|La poche du gilet garde une plume, collée au sac.</t>
         </is>
       </c>
@@ -6256,17 +6256,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet se touchent, chauds, devant le vide.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Deux tissus, et tu ne grelottes plus. Le manteau et le gilet se touchent, chauds, devant le vide.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet se touchent, chauds, devant le vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Deux tissus, et tu ne grelottes plus. Le manteau et le gilet se touchent, chauds, devant le vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet se touchent, chauds, devant le vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le manteau, deux chaleurs. Sur la chaise de la chambre, le linge s'est tu. À table, une goutte de lait fait un rond. Deux tissus, et tu ne grelottes plus. Le manteau et le gilet se touchent, chauds, devant le vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6405,7 +6405,7 @@
 enfant-f|J'ai mis le gilet, le manteau, deux chaleurs.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Deux tissus, et tu ne grelottes plus.
 narrateur|Le manteau et le gilet se touchent, chauds, devant le vide.</t>
         </is>
       </c>
@@ -6622,17 +6622,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'endort dans le gilet, le volet ouvert.</t>
+          <t>Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Ils se sont endormis dans la laine. Le doudou s'endort dans le gilet, le volet ouvert.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'endort dans le gilet, le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Ils se sont endormis dans la laine. Le doudou s'endort dans le gilet, le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'endort dans le gilet, le &lt;emphasis&gt;volet&lt;/emphasis&gt; ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Raconte, Victorina, on t'écoute. J'ai mis le gilet, le doudou dans la poche. Sur la chaise de la chambre, le linge s'est tu. À table, le moineau chante, trop loin pour le bol. Ils se sont endormis dans la laine. Le doudou s'endort dans le gilet, le &lt;emphasis&gt;volet&lt;/emphasis&gt; ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6775,7 +6775,7 @@
 enfant-f|J'ai mis le gilet, le doudou dans la poche.
 narrateur|Sur la chaise de la chambre, le linge s'est tu.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Ils se sont endormis dans la laine.
 narrateur|Le doudou s'endort dans le gilet, le volet ouvert.</t>
         </is>
       </c>
@@ -8129,17 +8129,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Dans le sac, l'oiseau sent le savon, et le vent.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tes mains ont tenu, sèches, cette fois. Dans le sac, l'oiseau sent le savon, et le vent.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Dans le sac, l'oiseau sent le savon, et le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tes mains ont tenu, sèches, cette fois. Dans le sac, l'oiseau sent le savon, et le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Dans le sac, l'oiseau sent le savon, et le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tes mains ont tenu, sèches, cette fois. Dans le sac, l'oiseau sent le savon, et le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8273,12 +8273,12 @@
       </c>
       <c r="AW39" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai séché mes mains, le t-shirt, le sac a pris l'oiseau.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Tes mains ont tenu, sèches, cette fois.
 narrateur|Dans le sac, l'oiseau sent le savon, et le vent.</t>
         </is>
       </c>
@@ -8495,17 +8495,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sèche une goutte, près de la poignée.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le manteau a bu la goutte, toi. Le manteau sèche une goutte, près de la poignée.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sèche une goutte, près de la poignée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le manteau a bu la goutte, toi. Le manteau sèche une goutte, près de la poignée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sèche une goutte, près de la poignée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le manteau a bu la goutte. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le manteau a bu la goutte, toi. Le manteau sèche une goutte, près de la poignée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8639,12 +8639,12 @@
       </c>
       <c r="AW41" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai séché, le t-shirt, le manteau a bu la goutte.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le manteau a bu la goutte, toi.
 narrateur|Le manteau sèche une goutte, près de la poignée.</t>
         </is>
       </c>
@@ -8861,17 +8861,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a les joues humides, et il rit vers la rue.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou n'a pas eu d'eau. Le doudou a les joues humides, et il rit vers la rue.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a les joues humides, et il rit vers la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou n'a pas eu d'eau. Le doudou a les joues humides, et il rit vers la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a les joues humides, et il rit vers la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai séché, le t-shirt, le doudou n'a pas eu d'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou n'a pas eu d'eau. Le doudou a les joues humides, et il rit vers la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9005,12 +9005,12 @@
       </c>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai séché, le t-shirt, le doudou n'a pas eu d'eau.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le doudou n'a pas eu d'eau.
 narrateur|Le doudou a les joues humides, et il rit vers la rue.</t>
         </is>
       </c>
@@ -9615,17 +9615,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette laisse une trace ronde, sous le sac.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La trace ronde, c'est ta chaussette. Une chaussette laisse une trace ronde, sous le sac.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette laisse une trace ronde, sous le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La trace ronde, c'est ta chaussette. Une chaussette laisse une trace ronde, sous le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Une chaussette laisse une trace ronde, sous le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes sèches, le sac sous la poignée. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La trace ronde, c'est ta chaussette. Une chaussette laisse une trace ronde, sous le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9759,12 +9759,12 @@
       </c>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis les chaussettes sèches, le sac sous la poignée.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|La trace ronde, c'est ta chaussette.
 narrateur|Une chaussette laisse une trace ronde, sous le sac.</t>
         </is>
       </c>
@@ -9981,17 +9981,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sent le savon, et la rue entre.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu es restée droite, près du bois. Le manteau sent le savon, et la rue entre.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sent le savon, et la rue entre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu es restée droite, près du bois. Le manteau sent le savon, et la rue entre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau sent le savon, et la rue entre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le manteau, sans sauter. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu es restée droite, près du bois. Le manteau sent le savon, et la rue entre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10125,12 +10125,12 @@
       </c>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis les chaussettes, le manteau, sans sauter.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Tu es restée droite, près du bois.
 narrateur|Le manteau sent le savon, et la rue entre.</t>
         </is>
       </c>
@@ -10347,17 +10347,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, les pieds au chaud, voit le moineau.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou a vu le moineau, au sec. Le doudou, les pieds au chaud, voit le moineau.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, les pieds au chaud, voit le moineau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou a vu le moineau, au sec. Le doudou, les pieds au chaud, voit le moineau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, les pieds au chaud, voit le moineau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis les chaussettes, le doudou loin des gouttes. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le doudou a vu le moineau, au sec. Le doudou, les pieds au chaud, voit le moineau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10491,12 +10491,12 @@
       </c>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis les chaussettes, le doudou loin des gouttes.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le doudou a vu le moineau, au sec.
 narrateur|Le doudou, les pieds au chaud, voit le moineau.</t>
         </is>
       </c>
@@ -10529,17 +10529,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le gilet, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton d'abord, la poignée ensuite. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?</t>
+          <t>Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le gilet, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton est ouvert, face au miroir. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton d'abord, la poignée ensuite. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton est ouvert, face au miroir. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton d'abord, la poignée ensuite. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Ses mains sentent le savon, plus sèches, plus prêtes. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, près de la buée. Je le mets, et je repars ! La laine accroche une goutte, trop pressée. Un bouton reste ouvert, face au miroir. Le bouton est ouvert, face au miroir. La laine mouillée pique, comme le savon. Il me tient le ventre, tout ouvert ! Elle s'arrête, et le bouton rentre, net. Le gilet sent le savon, et un peu de laine. Tes épaules sont prêtes, pour le bois. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10682,7 +10682,7 @@
 enfant-f|Je le mets, et je repars !
 narrateur|La laine accroche une goutte, trop pressée.
 narrateur|Un bouton reste ouvert, face au miroir.
-maman|Le bouton d'abord, la poignée ensuite.
+maman|Le bouton est ouvert, face au miroir.
 papa|La laine mouillée pique, comme le savon.
 enfant-f|Il me tient le ventre, tout ouvert !
 narrateur|Elle s'arrête, et le bouton rentre, net.
@@ -11100,17 +11100,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet sent le savon, près du sac.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La poche sent le savon, et le vent. La poche du gilet sent le savon, près du sac.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet sent le savon, près du sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La poche sent le savon, et le vent. La poche du gilet sent le savon, près du sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet sent le savon, près du sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le sac au sec, loin de l'eau. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le pain casse, tiède, sous les doigts. La poche sent le savon, et le vent. La poche du gilet sent le savon, près du sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11244,12 +11244,12 @@
       </c>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis le gilet, le sac au sec, loin de l'eau.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|La poche sent le savon, et le vent.
 narrateur|La poche du gilet sent le savon, près du sac.</t>
         </is>
       </c>
@@ -11465,17 +11465,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau boutonne le gilet, face au soleil.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le bouton du manteau a fait le reste. Le manteau boutonne le gilet, face au soleil.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau boutonne le gilet, face au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le bouton du manteau a fait le reste. Le manteau boutonne le gilet, face au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau boutonne le gilet, face au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le manteau a boutonné. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, une goutte de lait fait un rond. Le bouton du manteau a fait le reste. Le manteau boutonne le gilet, face au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11609,12 +11609,12 @@
       </c>
       <c r="AW57" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis le gilet, le manteau a boutonné.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le bouton du manteau a fait le reste.
 narrateur|Le manteau boutonne le gilet, face au soleil.</t>
         </is>
       </c>
@@ -11830,17 +11830,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'abrite dans le gilet, le bois ouvert.</t>
+          <t>Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le gilet a fait un toit, pour lui. Le doudou s'abrite dans le gilet, le bois ouvert.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'abrite dans le gilet, le bois ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le gilet a fait un toit, pour lui. Le doudou s'abrite dans le gilet, le bois ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou s'abrite dans le gilet, le bois ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, une miette roule vers le bol. Dis-nous, le pain est prêt. J'ai mis le gilet, le doudou sous le toit de laine. Dans la salle d'eau, le miroir n'a plus d'œil de buée. À table, le moineau chante, trop loin pour le bol. Le gilet a fait un toit, pour lui. Le doudou s'abrite dans le gilet, le bois ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -11974,12 +11974,12 @@
       </c>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, une miette roule vers le bol.
 maman|Dis-nous, le pain est prêt.
 enfant-f|J'ai mis le gilet, le doudou sous le toit de laine.
 narrateur|Dans la salle d'eau, le miroir n'a plus d'œil de buée.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le gilet a fait un toit, pour lui.
 narrateur|Le doudou s'abrite dans le gilet, le bois ouvert.</t>
         </is>
       </c>
@@ -12761,17 +12761,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le t-shirt, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bras d'abord, le bol ensuite. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?</t>
+          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le t-shirt, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bol est trop près, sors le bras. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis level="moderate"&gt;t-shirt&lt;/emphasis&gt;, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bras d'abord, le bol ensuite. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis level="moderate"&gt;t-shirt&lt;/emphasis&gt;, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bol est trop près, sors le bras. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis&gt;t-shirt&lt;/emphasis&gt;, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bras d'abord, le bol ensuite. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis&gt;t-shirt&lt;/emphasis&gt;, près du four. Je le mets, et je prends l'huile ! Elle enfile trop vite, le coton se tord. Une manche frôle le bol, trop près de l'huile. Le bol est trop près, sors le bras. Le pain dore, et toi, tu grelottes moins. La manche a failli tout tacher ! Elle ralentit, et le t-shirt tombe droit. Le coton garde un peu de chaleur du four. Avec ça, tu peux porter l'huile. J'ai le coton, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12914,7 +12914,7 @@
 enfant-f|Je le mets, et je prends l'huile !
 narrateur|Elle enfile trop vite, le coton se tord.
 narrateur|Une manche frôle le bol, trop près de l'huile.
-papa|Le bras d'abord, le bol ensuite.
+papa|Le bol est trop près, sors le bras.
 maman|Le pain dore, et toi, tu grelottes moins.
 enfant-f|La manche a failli tout tacher !
 narrateur|Elle ralentit, et le t-shirt tombe droit.
@@ -13333,17 +13333,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Le sac, près du bol, garde l'oiseau et une miette.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. L'huile a parlé au bois, sans bruit. Le sac, près du bol, garde l'oiseau et une miette.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Le sac, près du bol, garde l'oiseau et une miette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. L'huile a parlé au bois, sans bruit. Le sac, près du bol, garde l'oiseau et une miette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Le sac, près du bol, garde l'oiseau et une miette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le sac a l'huile et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. L'huile a parlé au bois, sans bruit. Le sac, près du bol, garde l'oiseau et une miette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13477,12 +13477,12 @@
       </c>
       <c r="AW67" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le t-shirt, le sac a l'huile et l'oiseau.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|L'huile a parlé au bois, sans bruit.
 narrateur|Le sac, près du bol, garde l'oiseau et une miette.</t>
         </is>
       </c>
@@ -13699,17 +13699,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près du pain, tient un fil de soleil.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le pain a vu la rue, avec toi. Le manteau, près du pain, tient un fil de soleil.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près du pain, tient un fil de soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le pain a vu la rue, avec toi. Le manteau, près du pain, tient un fil de soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, près du pain, tient un fil de soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le manteau, et le pain a vu la rue. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le pain a vu la rue, avec toi. Le manteau, près du pain, tient un fil de soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13843,12 +13843,12 @@
       </c>
       <c r="AW69" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le t-shirt, le manteau, et le pain a vu la rue.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le pain a vu la rue, avec toi.
 narrateur|Le manteau, près du pain, tient un fil de soleil.</t>
         </is>
       </c>
@@ -14065,17 +14065,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, près du four, regarde le volet ouvert.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a deux odeurs, le doudou. Le doudou, près du four, regarde le volet ouvert.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, près du four, regarde le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a deux odeurs, le doudou. Le doudou, près du four, regarde le &lt;emphasis level="moderate"&gt;volet&lt;/emphasis&gt; ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, près du four, regarde le &lt;emphasis&gt;volet&lt;/emphasis&gt; ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le t-shirt, le doudou a le four et la rue. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a deux odeurs, le doudou. Le doudou, près du four, regarde le &lt;emphasis&gt;volet&lt;/emphasis&gt; ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14213,12 +14213,12 @@
       </c>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le t-shirt, le doudou a le four et la rue.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Il a deux odeurs, le doudou.
 narrateur|Le doudou, près du four, regarde le volet ouvert.</t>
         </is>
       </c>
@@ -14251,17 +14251,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les chaussettes, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Le talon d'abord, l'huile ensuite. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?</t>
+          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les chaussettes, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Ton talon est plié, l'huile attend. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les &lt;emphasis level="moderate"&gt;chaussettes&lt;/emphasis&gt;, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Le talon d'abord, l'huile ensuite. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les &lt;emphasis level="moderate"&gt;chaussettes&lt;/emphasis&gt;, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Ton talon est plié, l'huile attend. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les &lt;emphasis&gt;chaussettes&lt;/emphasis&gt;, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Le talon d'abord, l'huile ensuite. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend les &lt;emphasis&gt;chaussettes&lt;/emphasis&gt;, sous la table. Je les mets, et je prends l'huile ! Elle enfile trop vite, un talon reste plié. Sur les carreaux, le talon plié la fait pencher. Ton talon est plié, l'huile attend. Les carreaux piquent moins, avec ça. Mon talon me chatouille ! Elle s'assoit, et le talon se déplie, net. Les deux chaussettes tiennent, chaudes, sous la table. Avec ça, tu peux porter l'huile. J'ai les deux, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14404,7 +14404,7 @@
 enfant-f|Je les mets, et je prends l'huile !
 narrateur|Elle enfile trop vite, un talon reste plié.
 narrateur|Sur les carreaux, le talon plié la fait pencher.
-papa|Le talon d'abord, l'huile ensuite.
+papa|Ton talon est plié, l'huile attend.
 maman|Les carreaux piquent moins, avec ça.
 enfant-f|Mon talon me chatouille !
 narrateur|Elle s'assoit, et le talon se déplie, net.
@@ -14822,17 +14822,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Les chaussettes, sous la table, sentent le pain chaud.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Les carreaux n'ont plus piqué tes pieds. Les chaussettes, sous la table, sentent le pain chaud.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Les chaussettes, sous la table, sentent le pain chaud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Les carreaux n'ont plus piqué tes pieds. Les chaussettes, sous la table, sentent le pain chaud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. Les chaussettes, sous la table, sentent le pain chaud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le sac près du bol. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Les carreaux n'ont plus piqué tes pieds. Les chaussettes, sous la table, sentent le pain chaud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -14966,12 +14966,12 @@
       </c>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis les chaussettes, le sac près du bol.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Les carreaux n'ont plus piqué tes pieds.
 narrateur|Les chaussettes, sous la table, sentent le pain chaud.</t>
         </is>
       </c>
@@ -15188,17 +15188,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, sur la chaise de cuisine, garde le vent.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le manteau gardera le vent, en bas. Le manteau, sur la chaise de cuisine, garde le vent.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, sur la chaise de cuisine, garde le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le manteau gardera le vent, en bas. Le manteau, sur la chaise de cuisine, garde le vent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau, sur la chaise de cuisine, garde le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le manteau, pour le pain dehors. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le manteau gardera le vent, en bas. Le manteau, sur la chaise de cuisine, garde le vent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15332,12 +15332,12 @@
       </c>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis les chaussettes, le manteau, pour le pain dehors.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le manteau gardera le vent, en bas.
 narrateur|Le manteau, sur la chaise de cuisine, garde le vent.</t>
         </is>
       </c>
@@ -15553,17 +15553,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a une miette sur le nez, et la rue.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a une miette, et la rue. Le doudou a une miette sur le nez, et la rue.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a une miette sur le nez, et la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a une miette, et la rue. Le doudou a une miette sur le nez, et la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou a une miette sur le nez, et la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis les chaussettes, le doudou a une miette. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il a une miette, et la rue. Le doudou a une miette sur le nez, et la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15697,12 +15697,12 @@
       </c>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis les chaussettes, le doudou a une miette.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Il a une miette, et la rue.
 narrateur|Le doudou a une miette sur le nez, et la rue.</t>
         </is>
       </c>
@@ -15735,17 +15735,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le gilet, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche d'abord, le bol ensuite. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?</t>
+          <t>L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le gilet, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche est à l'envers, loin du bol. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche d'abord, le bol ensuite. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis level="moderate"&gt;gilet&lt;/emphasis&gt;, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche est à l'envers, loin du bol. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche d'abord, le bol ensuite. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;L'odeur du pain suit ses pas, jusque sous le bois. Victorina prend le &lt;emphasis&gt;gilet&lt;/emphasis&gt;, près du four tiède. Je le mets, et je prends l'huile ! Elle enfile trop vite, la poche se retourne. L'huile frôle la laine, trop près du bol. La poche est à l'envers, loin du bol. La laine tiédit, comme le pain. La poche voulait tout avaler ! Elle la remet, sans toucher l'huile. Le gilet ferme, et une poche attend, nette. Avec ça, tu peux porter l'huile. J'ai la laine, et après ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15888,7 +15888,7 @@
 enfant-f|Je le mets, et je prends l'huile !
 narrateur|Elle enfile trop vite, la poche se retourne.
 narrateur|L'huile frôle la laine, trop près du bol.
-papa|La poche d'abord, le bol ensuite.
+papa|La poche est à l'envers, loin du bol.
 maman|La laine tiédit, comme le pain.
 enfant-f|La poche voulait tout avaler !
 narrateur|Elle la remet, sans toucher l'huile.
@@ -16306,17 +16306,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet tient une miette, et l'oiseau.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. La poche a fait le voyage, toi. La poche du gilet tient une miette, et l'oiseau.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet tient une miette, et l'oiseau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. La poche a fait le voyage, toi. La poche du gilet tient une miette, et l'oiseau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. Tu as ouvert, sans tout tirer d'un coup. La poche du gilet tient une miette, et l'oiseau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le sac a une miette et l'oiseau. Sur la table, le pain fume, une miette à part. À table, le pain casse, tiède, sous les doigts. La poche a fait le voyage, toi. La poche du gilet tient une miette, et l'oiseau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16450,12 +16450,12 @@
       </c>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le gilet, le sac a une miette et l'oiseau.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le pain casse, tiède, sous les doigts.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|La poche a fait le voyage, toi.
 narrateur|La poche du gilet tient une miette, et l'oiseau.</t>
         </is>
       </c>
@@ -16671,17 +16671,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet, près du four, sentent le pain.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le four a prêté sa chaleur. Le manteau et le gilet, près du four, sentent le pain.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet, près du four, sentent le pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le four a prêté sa chaleur. Le manteau et le gilet, près du four, sentent le pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Tu as ouvert, sans tout tirer d'un coup. Le manteau et le gilet, près du four, sentent le pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le manteau, on sentait le four. Sur la table, le pain fume, une miette à part. À table, une goutte de lait fait un rond. Le four a prêté sa chaleur. Le manteau et le gilet, près du four, sentent le pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16815,12 +16815,12 @@
       </c>
       <c r="AW85" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le gilet, le manteau, on sentait le four.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, une goutte de lait fait un rond.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Le four a prêté sa chaleur.
 narrateur|Le manteau et le gilet, près du four, sentent le pain.</t>
         </is>
       </c>
@@ -17036,17 +17036,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, dans le gilet, écoute le moineau, loin.</t>
+          <t>Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il écoute le moineau, sans crier. Le doudou, dans le gilet, écoute le moineau, loin.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, dans le gilet, écoute le moineau, loin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il écoute le moineau, sans crier. Le doudou, dans le gilet, écoute le moineau, loin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, tout chaud. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Tu as ouvert, sans tout tirer d'un coup. Le doudou, dans le gilet, écoute le moineau, loin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le four s'est tu, et le pain fume. À toi, on a fini nos phrases. J'ai mis le gilet, le doudou écoute le moineau. Sur la table, le pain fume, une miette à part. À table, le moineau chante, trop loin pour le bol. Il écoute le moineau, sans crier. Le doudou, dans le gilet, écoute le moineau, loin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17180,12 +17180,12 @@
       </c>
       <c r="AW87" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, le pain est sur la table, tout chaud.
+          <t>narrateur|Plus tard, le four s'est tu, et le pain fume.
 maman|À toi, on a fini nos phrases.
 enfant-f|J'ai mis le gilet, le doudou écoute le moineau.
 narrateur|Sur la table, le pain fume, une miette à part.
 narrateur|À table, le moineau chante, trop loin pour le bol.
-papa|Tu as ouvert, sans tout tirer d'un coup.
+papa|Il écoute le moineau, sans crier.
 narrateur|Le doudou, dans le gilet, écoute le moineau, loin.</t>
         </is>
       </c>
@@ -17212,7 +17212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17283,6 +17283,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>